<commit_message>
check-package PASS, and the derived layer rebuilt clean
First run this session with no errors anywhere except the three authored
inputs, which need a walk rather than a tool. check-screens, check-states,
check-traceability, check-board-flows, check-wireframes, check-migrations,
check-flows, check-frontend, check-config-scope, check-lineage and every audit
pass; transition coverage holds at 95%.

The numbers the fixes were meant to move: lineage 1,974 against 1,974 contract
operations, 561 tables with no retail.wallet orphan returning, 1,189
relationship edges and 984 column references where there were 955.

Coverage reads 91.1% surfaced by a screen, 0.7% machine-called and complete,
91.7% accounted for, 8.3% with no surface yet.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>platform, workforce, approvals</t>
+          <t>platform, workforce, approvals, accreditation, tenancy</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>orders</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>queue, maintenance, resources, venuemap, assets, games</t>
+          <t>queue, maintenance, resources, venuemap, assets, games, rental</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>control, subscription</t>
         </is>
       </c>
       <c r="H19" s="10" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C20" s="10" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VenueOpsService</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PlatformService</t>
         </is>
       </c>
       <c r="C30" s="10" t="n">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C32" s="10" t="n">
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -3068,7 +3068,7 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Block A in OpenProject, and the package it points at made to match its own standards
OpenProject: push-openproject.py creates tickets with full descriptions (op-descriptions.py) and
leaves the 1,770 "follows" links to a server-side run (op-bulk-links.*), since OpenProject 10
re-walks its graph per API link. adam-links.py builds ADAM's ticket links. Runbook:
handoff/service-docs/OPENPROJECT-PUSH.md.

Standards, from the #20354 review (action register N5-N10):
- scope_path and every *_scope_path is ltree with GiST indexes; in_scope no longer casts
- 27 money columns say gross, net or list price, via x-ticvai-column; API names unchanged
- shared errors are implicit (api-conventions 5); venues do not see tenant-level rows (5.3)
- venue_in_scope shows tenant-level rows to a tenant-root grant only, and hides them if a
  database ever holds two tenants; the control database carries no venue functions

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>32</v>
@@ -756,10 +756,10 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
@@ -1047,10 +1047,10 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
@@ -1191,10 +1191,10 @@
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>13</v>
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="C21" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D21" s="10" t="n">
         <v>20</v>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="C18" s="10" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>white-label</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr"/>
@@ -2682,7 +2682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
@@ -3286,21 +3286,21 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>wallet.wallet_transaction</t>
+          <t>orders.cart</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>WalletService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>orders, wallet</t>
+          <t>marketing-crm, orders</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
@@ -3311,17 +3311,17 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>catalogue.product_version</t>
+          <t>wallet.wallet_transaction</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>WalletService</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>catalogue, fnb</t>
+          <t>orders, wallet</t>
         </is>
       </c>
       <c r="D28" s="10" t="n">
@@ -3336,21 +3336,21 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>payments.routing_rule</t>
+          <t>catalogue.product_version</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>orders, payments</t>
+          <t>catalogue, fnb</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -3361,17 +3361,17 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>catalogue.price</t>
+          <t>payments.routing_rule</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>fnb, inventory</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="D30" s="10" t="n">
@@ -3386,23 +3386,48 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>platform.audit_record</t>
+          <t>catalogue.price</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>inventory, tenancy</t>
+          <t>fnb, inventory</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>platform.audit_record</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>TenancyService</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>inventory, tenancy</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>

</xml_diff>

<commit_message>
TICVAI: release refresh for r1 (refresh-safe passed)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -756,10 +756,10 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
@@ -1288,10 +1288,10 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>finance, inventory, orders, payments, tenancy</t>
+          <t>finance, inventory, orders, payments, platform-ops, tenancy</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TICVAI: refresh for r1 of the fresh start (refresh-safe PASS on b23001f6: the four spec-fix branches and the gate fixes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>114</v>
@@ -999,10 +999,10 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>51</v>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D17" s="10" t="n">
         <v>132</v>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="C18" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TICVAI r2: release refresh (refresh-safe PASS on cbb7e421: kiosk customisation, BOCA, Block A2 plan, the r4-batch fixes, mirrors)
refresh-safe run 20261006-172054-17266: 70 checkers, 0 gate failures; baseline-known only (check-package 2,
check-authored-inputs 7, check-screen-patterns 12 pinned); 43 added, 935 modified, 0 deleted under ticvai/.
Adds the tenant forward migration V0100__after_r1_20261006.sql (the five whitelabel.kiosk_* tables).

CHG-exempt: release refresh

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -1337,10 +1337,10 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="C38" s="10" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TICVAI r2: release refresh (refresh-safe PASS on 0f44e75c: 71 checkers, 0 gate failures) with the package defect fixes (CHG-R4-011..016), the client's tracker answers (CHG-R4-017..019), the BOCA addresses, the forward migration V0101 and the six mirrors
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>115</v>
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
TICVAI r4: derived output of the passing gate (refresh-safe --parallel 4 on c39a2695: 75 checkers, 0 gate failures; derive 19m56s); forward migration V0102__after_r1_20261013 (11 columns, 13 indexes, additive); the plan with Pallavi Sawant's back end moved and the back-end pace at 7 a day; mirrors
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>138</v>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>77</v>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D17" s="10" t="n">
         <v>132</v>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>catalogue, fnb, inventory, orders, payments, venue-map</t>
+          <t>catalogue, inventory, orders, payments, venue-map</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>access, ai, finance, games, marketing-crm, promotions +4</t>
+          <t>access, ai, finance, fnb, games, marketing-crm +5</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1771,12 +1771,12 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>approvals, finance, marketing-crm, platform-ops, public-api, subscription, tenancy, white-label</t>
+          <t>approvals, marketing-crm, platform-ops, public-api, subscription, tenancy, white-label</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>ai, finance</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>access, accreditation, approvals, catalogue, cross-region, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, seating, shift, subscription, tenancy, wallet, white-label</t>
+          <t>access, accreditation, approvals, catalogue, cross-region, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -2744,7 +2744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, seating, shift, subscription, tenancy, wallet, white-label</t>
+          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>catalogue.inventory_hold</t>
+          <t>catalogue.inventory_reservation</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -3198,7 +3198,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>inventory.stock_reservation</t>
+          <t>inventory.stock_earmark</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -3298,7 +3298,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>catalogue.price</t>
+          <t>catalogue.product</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>catalogue, fnb, inventory</t>
+          <t>catalogue, inventory</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>catalogue.product</t>
+          <t>platform.region_settings</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>catalogue, inventory</t>
+          <t>finance, tenancy</t>
         </is>
       </c>
       <c r="D26" s="10" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>platform.region_settings</t>
+          <t>orders.order_event</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>finance, tenancy</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>orders.order_event</t>
+          <t>promotions.promotion_evaluation_trace</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>orders, payments</t>
+          <t>orders, promotions</t>
         </is>
       </c>
       <c r="D28" s="10" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>promotions.promotion_evaluation_trace</t>
+          <t>orders.refund</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>orders, promotions</t>
+          <t>orders, wallet</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>orders.refund</t>
+          <t>payments.payment_attempt</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>orders, wallet</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="D30" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>payments.payment_attempt</t>
+          <t>ledger.price_variance</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>LedgerService</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>orders, payments</t>
+          <t>finance, orders</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>ledger.price_variance</t>
+          <t>platform.dsar_request</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>LedgerService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>finance, orders</t>
+          <t>cross-region, identity</t>
         </is>
       </c>
       <c r="D32" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>platform.dsar_request</t>
+          <t>identity.role_permission</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>IdentityService</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>cross-region, identity</t>
+          <t>identity, tenancy</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>identity.role_permission</t>
+          <t>identity.delegated_access</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
@@ -3533,22 +3533,22 @@
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>identity, tenancy</t>
+          <t>identity, orders</t>
         </is>
       </c>
       <c r="D34" s="10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>A share and a developer membership are both delegated authority (CF-132) — one mechanism, three callers.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>identity.delegated_access</t>
+          <t>pii.subject</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -3558,61 +3558,61 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>identity, orders</t>
+          <t>identity, marketing-crm</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>A share and a developer membership are both delegated authority (CF-132) — one mechanism, three callers.</t>
+          <t>**`identity` is the only real writer.** `marketing-crm` updates a profile field the subject owns — and consent never merges permissively (CF-160).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>pii.subject</t>
+          <t>seating.seat_reservation</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>IdentityService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>identity, marketing-crm</t>
+          <t>catalogue, seating</t>
         </is>
       </c>
       <c r="D36" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>**`identity` is the only real writer.** `marketing-crm` updates a profile field the subject owns — and consent never merges permissively (CF-160).</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>control.invoice_line</t>
+          <t>inventory.count_line</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>PlatformService</t>
+          <t>InventoryService</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>finance, subscription</t>
+          <t>fnb, inventory</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
@@ -3623,17 +3623,17 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>seating.seat_hold</t>
+          <t>inventory.requisition</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>InventoryService</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>catalogue, seating</t>
+          <t>inventory, maintenance</t>
         </is>
       </c>
       <c r="D38" s="10" t="n">
@@ -3648,21 +3648,21 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>inventory.count_line</t>
+          <t>wallet.wallet_transaction</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>InventoryService</t>
+          <t>WalletService</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>fnb, inventory</t>
+          <t>orders, wallet</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>inventory.requisition</t>
+          <t>maintenance.asset</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>InventoryService</t>
+          <t>VenueOpsService</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>inventory, maintenance</t>
+          <t>maintenance, rental</t>
         </is>
       </c>
       <c r="D40" s="10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
@@ -3698,32 +3698,32 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>wallet.wallet_transaction</t>
+          <t>ai.activity</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>WalletService</t>
+          <t>AiService</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>orders, wallet</t>
+          <t>ai, reporting</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>**The governed reporting pair** (ADR-0020). `reporting` may write an AI interaction because a natural-language query is one.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>maintenance.asset</t>
+          <t>games.card</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>maintenance, rental</t>
+          <t>games, wallet</t>
         </is>
       </c>
       <c r="D42" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
@@ -3748,46 +3748,46 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>ai.activity</t>
+          <t>control.partner_agreement</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>AiService</t>
+          <t>PlatformService</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>ai, reporting</t>
+          <t>approvals, subscription</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>**The governed reporting pair** (ADR-0020). `reporting` may write an AI interaction because a natural-language query is one.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>games.card</t>
+          <t>control.partner_application</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>VenueOpsService</t>
+          <t>PlatformService</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>games, wallet</t>
+          <t>approvals, subscription</t>
         </is>
       </c>
       <c r="D44" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>control.partner_agreement</t>
+          <t>control.partner_change_request</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>control.partner_application</t>
+          <t>marketing.privacy_notice_governance</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>PlatformService</t>
+          <t>MarketingService</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>approvals, subscription</t>
+          <t>approvals, marketing-crm</t>
         </is>
       </c>
       <c r="D46" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>control.partner_change_request</t>
+          <t>orders.cart_line</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>PlatformService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>approvals, subscription</t>
+          <t>orders, venue-map</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
@@ -3873,17 +3873,17 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>marketing.privacy_notice_governance</t>
+          <t>payments.routing_rule</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>MarketingService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>approvals, marketing-crm</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="D48" s="10" t="n">
@@ -3898,21 +3898,21 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>orders.cart_line</t>
+          <t>catalogue.price</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>orders, venue-map</t>
+          <t>catalogue, inventory</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>catalogue.product_version</t>
+          <t>seating.seat_reservation_item</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>catalogue, fnb</t>
+          <t>catalogue, seating</t>
         </is>
       </c>
       <c r="D50" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
@@ -3948,73 +3948,23 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>payments.routing_rule</t>
+          <t>tenancy.data_retention_setting</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>orders, payments</t>
+          <t>access, tenancy</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>seating.seat_hold_item</t>
-        </is>
-      </c>
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t>CatalogueService</t>
-        </is>
-      </c>
-      <c r="C52" s="10" t="inlineStr">
-        <is>
-          <t>catalogue, seating</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>tenancy.data_retention_setting</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>TenancyService</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
-        <is>
-          <t>access, tenancy</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>

</xml_diff>

<commit_message>
Audit base, derived: the full derive of dfdc3388 (14 Oct), so every audit fix branch starts from a derived package; not a release
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>cross-region, identity, marketing-crm, reporting, subscription, tenancy +2</t>
+          <t>cross-region, marketing-crm, reporting, subscription, tenancy, venue-map +1</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>approvals, subscription, workforce</t>
+          <t>approvals, finance, identity, subscription, workforce</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>access, ai, finance, fnb, games, marketing-crm +5</t>
+          <t>access, ai, finance, fnb, games, marketing-crm +6</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>access, ai, catalogue, finance, promotions</t>
+          <t>access, ai, catalogue, finance, promotions, tenancy</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>access, accreditation, approvals, catalogue, cross-region, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
+          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
@@ -2521,12 +2521,12 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>access, games, orders, subscription</t>
+          <t>access, cross-region, games, orders, subscription</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>cross-region</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2744,7 +2744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
+          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -2848,71 +2848,71 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>marketing.message_dispatch</t>
+          <t>platform.audit_record</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>MarketingService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>fnb, identity, marketing-crm, orders, public-api, workforce</t>
+          <t>finance, identity, inventory, orders, payments, platform-ops, tenancy</t>
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>**Five writers, and every one is sending a message somebody asked for.** A verification email, a payment link, an evacuation notice.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>platform.audit_record</t>
+          <t>marketing.message_dispatch</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>MarketingService</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>finance, inventory, orders, payments, platform-ops, tenancy</t>
+          <t>fnb, identity, marketing-crm, orders, public-api, workforce</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>**Five writers, and every one is sending a message somebody asked for.** A verification email, a payment link, an evacuation notice.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>catalogue.inventory_reservation</t>
+          <t>sync.rejection</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>CrossRegionService</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>catalogue, orders, payments, venue-map</t>
+          <t>access, cross-region, games, orders, subscription</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>orders.payment</t>
+          <t>approvals.request</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>orders, payments, subscription, wallet</t>
+          <t>approvals, finance, identity, subscription, workforce</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
@@ -2948,46 +2948,46 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>ledger.journal_entry</t>
+          <t>catalogue.inventory_reservation</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>LedgerService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>finance, orders, payments, shift</t>
+          <t>catalogue, orders, payments, venue-map</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>As above. The journal is written by whatever caused the money to move.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>sync.rejection</t>
+          <t>orders.payment</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>CrossRegionService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>access, games, orders, subscription</t>
+          <t>orders, payments, subscription, wallet</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
@@ -2998,107 +2998,107 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>inventory.movement</t>
+          <t>ledger.journal_entry</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>InventoryService</t>
+          <t>LedgerService</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>fnb, inventory, maintenance, retail</t>
+          <t>finance, orders, payments, shift</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>**Every stock change is a movement.** Waste from F&amp;B and adjustment from inventory are the same act with a different reason.</t>
+          <t>As above. The journal is written by whatever caused the money to move.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>catalogue.channel_capacity</t>
+          <t>inventory.movement</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>InventoryService</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>catalogue, orders, payments</t>
+          <t>fnb, inventory, maintenance, retail</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>**Every stock change is a movement.** Waste from F&amp;B and adjustment from inventory are the same act with a different reason.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>access.entitlement</t>
+          <t>catalogue.channel_capacity</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>AccessService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>access, catalogue, orders</t>
+          <t>catalogue, orders, payments</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>**A sale issues a ticket.** `orders` appends the entitlement, `catalogue` suspends and freezes it against its template. Neither redefines the row.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>orders.order_line</t>
+          <t>access.entitlement</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>AccessService</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>fnb, orders, subscription</t>
+          <t>access, catalogue, orders</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>**A sale issues a ticket.** `orders` appends the entitlement, `catalogue` suspends and freezes it against its template. Neither redefines the row.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>orders.sales_order</t>
+          <t>orders.order_line</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -3108,47 +3108,47 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>identity, orders, subscription</t>
+          <t>fnb, orders, subscription</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>`identity` links a guest checkout to an existing order. One field, on claim.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>ledger.posting</t>
+          <t>orders.sales_order</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>LedgerService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>finance, orders, shift</t>
+          <t>identity, orders, subscription</t>
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>**A till closing is a ledger act.** Settling a shift posts to the ledger, and a payment writes its own entry — appending, never redefining.</t>
+          <t>`identity` links a guest checkout to an existing order. One field, on claim.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>ledger.journal_line</t>
+          <t>ledger.posting</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -3158,36 +3158,36 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>finance, orders, payments</t>
+          <t>finance, orders, shift</t>
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>**A till closing is a ledger act.** Settling a shift posts to the ledger, and a payment writes its own entry — appending, never redefining.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>marketing.consent_record</t>
+          <t>ledger.journal_line</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>MarketingService</t>
+          <t>LedgerService</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>access, marketing-crm, orders</t>
+          <t>finance, orders, payments</t>
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>inventory.stock_earmark</t>
+          <t>marketing.consent_record</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>InventoryService</t>
+          <t>MarketingService</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>inventory, maintenance, retail</t>
+          <t>access, marketing-crm, orders</t>
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>approvals.request</t>
+          <t>inventory.stock_earmark</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>InventoryService</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>approvals, subscription, workforce</t>
+          <t>inventory, maintenance, retail</t>
         </is>
       </c>
       <c r="D22" s="10" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
@@ -3473,25 +3473,25 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>platform.dsar_request</t>
+          <t>identity.delegated_access</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>IdentityService</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>cross-region, identity</t>
+          <t>identity, orders</t>
         </is>
       </c>
       <c r="D32" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>A share and a developer membership are both delegated authority (CF-132) — one mechanism, three callers.</t>
         </is>
       </c>
     </row>
@@ -3523,7 +3523,7 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>identity.delegated_access</t>
+          <t>pii.subject</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
@@ -3533,61 +3533,61 @@
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>identity, orders</t>
+          <t>identity, marketing-crm</t>
         </is>
       </c>
       <c r="D34" s="10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>A share and a developer membership are both delegated authority (CF-132) — one mechanism, three callers.</t>
+          <t>**`identity` is the only real writer.** `marketing-crm` updates a profile field the subject owns — and consent never merges permissively (CF-160).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>pii.subject</t>
+          <t>seating.seat_reservation</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>IdentityService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>identity, marketing-crm</t>
+          <t>catalogue, seating</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>**`identity` is the only real writer.** `marketing-crm` updates a profile field the subject owns — and consent never merges permissively (CF-160).</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>seating.seat_reservation</t>
+          <t>inventory.count_line</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>InventoryService</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>catalogue, seating</t>
+          <t>fnb, inventory</t>
         </is>
       </c>
       <c r="D36" s="10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>inventory.count_line</t>
+          <t>inventory.requisition</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>fnb, inventory</t>
+          <t>inventory, maintenance</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>inventory.requisition</t>
+          <t>wallet.wallet_transaction</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>InventoryService</t>
+          <t>WalletService</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>inventory, maintenance</t>
+          <t>orders, wallet</t>
         </is>
       </c>
       <c r="D38" s="10" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>wallet.wallet_transaction</t>
+          <t>maintenance.asset</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>WalletService</t>
+          <t>VenueOpsService</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>orders, wallet</t>
+          <t>maintenance, rental</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
@@ -3673,71 +3673,71 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>maintenance.asset</t>
+          <t>ai.activity</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>VenueOpsService</t>
+          <t>AiService</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>maintenance, rental</t>
+          <t>ai, reporting</t>
         </is>
       </c>
       <c r="D40" s="10" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>**The governed reporting pair** (ADR-0020). `reporting` may write an AI interaction because a natural-language query is one.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>ai.activity</t>
+          <t>games.card</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>AiService</t>
+          <t>VenueOpsService</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>ai, reporting</t>
+          <t>games, wallet</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>**The governed reporting pair** (ADR-0020). `reporting` may write an AI interaction because a natural-language query is one.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>games.card</t>
+          <t>control.partner_agreement</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>VenueOpsService</t>
+          <t>PlatformService</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>games, wallet</t>
+          <t>approvals, subscription</t>
         </is>
       </c>
       <c r="D42" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>control.partner_agreement</t>
+          <t>control.partner_application</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -3762,7 +3762,7 @@
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>control.partner_application</t>
+          <t>control.partner_change_request</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D44" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
@@ -3798,17 +3798,17 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>control.partner_change_request</t>
+          <t>marketing.privacy_notice_governance</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>PlatformService</t>
+          <t>MarketingService</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>approvals, subscription</t>
+          <t>approvals, marketing-crm</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
@@ -3823,21 +3823,21 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>marketing.privacy_notice_governance</t>
+          <t>orders.cart_line</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>MarketingService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>approvals, marketing-crm</t>
+          <t>orders, venue-map</t>
         </is>
       </c>
       <c r="D46" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
@@ -3848,7 +3848,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>orders.cart_line</t>
+          <t>payments.routing_rule</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -3858,11 +3858,11 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>orders, venue-map</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
@@ -3873,17 +3873,17 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>payments.routing_rule</t>
+          <t>catalogue.price</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>orders, payments</t>
+          <t>catalogue, inventory</t>
         </is>
       </c>
       <c r="D48" s="10" t="n">
@@ -3898,17 +3898,17 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>catalogue.price</t>
+          <t>platform.dead_letter</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>catalogue, inventory</t>
+          <t>platform-ops, tenancy</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
@@ -3965,6 +3965,31 @@
         <v>2</v>
       </c>
       <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>pii.consent_identifier</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>IdentityService</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>identity, marketing-crm</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
         <is>
           <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>

</xml_diff>

<commit_message>
r8, derived: the final full derive of cd646999 (the walk fixes, the database update tasks, the gate fixes), from refresh-safe run 20261020-205348-305 (70 of 70 steps); gate judged only the started-ticket acknowledgements and check-ticket-builds' file links (fixed in 67435f71)
CHG-exempt: release refresh commit (derived output only; contracts changed only in their generated x-ticvai-consumed-by and screen-count annotations)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -1811,7 +1811,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>ai, inventory, promotions</t>
+          <t>ai, inventory, promotions, reporting</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>catalogue, inventory, subscription</t>
+          <t>catalogue, inventory, reporting, subscription</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>ai, catalogue, promotions, queue, resources, white-label</t>
+          <t>ai, catalogue, promotions, queue, reporting, resources +1</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>access, ai, catalogue, finance, promotions, tenancy</t>
+          <t>access, ai, catalogue, finance, promotions, reporting +1</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
r10, derived: the full derive of 3d11e6f6 (refresh-safe run 20261026-195338-1783, 72 of 72 steps; gate PASS with no failure outside tools/refresh-safe-baseline.json)
Forward migrations V0116 (control and tenant) and V0117 (names); the six mirrors; design batches, diagrams,
service docs and wireframes as the merged generators write them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
+++ b/ticvai/handoff/TICVAI_Services_and_Data_Segregation.xlsx
@@ -661,7 +661,7 @@
         <v>214</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>77</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D13" s="10" t="n">
         <v>127</v>
@@ -1288,10 +1288,10 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         <v>110</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>catalogue, inventory, orders, payments, venue-map</t>
+          <t>catalogue, inventory, orders, payments, promotions, venue-map</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>access, ai, finance, fnb, games, marketing-crm +6</t>
+          <t>access, ai, finance, fnb, games, marketing-crm +5</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="C20" s="10" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>fnb, identity, marketing-crm, orders, payments, resources, shift, subscription, venue-map, wallet</t>
+          <t>fnb, marketing-crm, orders, payments, resources, shift, subscription, venue-map, wallet</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
+          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, platform-ops, promotions, queue, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="C38" s="10" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
@@ -2744,7 +2744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, promotions, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
+          <t>access, accreditation, approvals, catalogue, finance, fnb, identity, inventory, maintenance, marketing-crm, orders, payments, promotions, queue, reporting, seating, shift, subscription, tenancy, wallet, white-label</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>catalogue.channel_capacity</t>
+          <t>catalogue.product</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>catalogue, orders, payments</t>
+          <t>catalogue, inventory, promotions</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
@@ -3048,57 +3048,57 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>access.entitlement</t>
+          <t>catalogue.channel_capacity</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>AccessService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>access, catalogue, orders</t>
+          <t>catalogue, orders, payments</t>
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>**A sale issues a ticket.** `orders` appends the entitlement, `catalogue` suspends and freezes it against its template. Neither redefines the row.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>orders.order_line</t>
+          <t>access.entitlement</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>AccessService</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>fnb, orders, subscription</t>
+          <t>access, catalogue, orders</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>**A sale issues a ticket.** `orders` appends the entitlement, `catalogue` suspends and freezes it against its template. Neither redefines the row.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>orders.sales_order</t>
+          <t>orders.order_line</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -3108,15 +3108,15 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>identity, orders, subscription</t>
+          <t>fnb, orders, subscription</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>`identity` links a guest checkout to an existing order. One field, on claim.</t>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>
       </c>
     </row>
@@ -3298,21 +3298,21 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>catalogue.product</t>
+          <t>platform.region_settings</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>catalogue, inventory</t>
+          <t>finance, tenancy</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>platform.region_settings</t>
+          <t>orders.order_event</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>finance, tenancy</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="D26" s="10" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>orders.order_event</t>
+          <t>orders.sales_order</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -3358,15 +3358,15 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>orders, payments</t>
+          <t>orders, subscription</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Checked and correct — a side effect of the writing service's own job.</t>
+          <t>`identity` links a guest checkout to an existing order. One field, on claim.</t>
         </is>
       </c>
     </row>
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D30" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>games.card</t>
+          <t>catalogue.variant</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>VenueOpsService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>games, wallet</t>
+          <t>catalogue, promotions</t>
         </is>
       </c>
       <c r="D42" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>control.partner_agreement</t>
+          <t>games.card</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>PlatformService</t>
+          <t>VenueOpsService</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>approvals, subscription</t>
+          <t>games, wallet</t>
         </is>
       </c>
       <c r="D43" s="7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>control.partner_application</t>
+          <t>control.partner_agreement</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D44" s="10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>control.partner_change_request</t>
+          <t>control.partner_application</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
@@ -3823,17 +3823,17 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>marketing.privacy_notice_governance</t>
+          <t>control.partner_change_request</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>MarketingService</t>
+          <t>PlatformService</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>approvals, marketing-crm</t>
+          <t>approvals, subscription</t>
         </is>
       </c>
       <c r="D46" s="10" t="n">
@@ -3848,21 +3848,21 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>approvals.matrix</t>
+          <t>marketing.privacy_notice_governance</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>MarketingService</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>approvals, white-label</t>
+          <t>approvals, marketing-crm</t>
         </is>
       </c>
       <c r="D47" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>orders.cart_line</t>
+          <t>approvals.matrix</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>OrderService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>orders, venue-map</t>
+          <t>approvals, white-label</t>
         </is>
       </c>
       <c r="D48" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>payments.routing_rule</t>
+          <t>orders.cart_line</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>orders, payments</t>
+          <t>orders, venue-map</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
@@ -3923,17 +3923,17 @@
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>catalogue.price</t>
+          <t>payments.routing_rule</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>OrderService</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>catalogue, inventory</t>
+          <t>orders, payments</t>
         </is>
       </c>
       <c r="D50" s="10" t="n">
@@ -3948,17 +3948,17 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>platform.dead_letter</t>
+          <t>catalogue.price</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>platform-ops, tenancy</t>
+          <t>catalogue, inventory</t>
         </is>
       </c>
       <c r="D51" s="7" t="n">
@@ -3973,17 +3973,17 @@
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>seating.seat_reservation_item</t>
+          <t>platform.dead_letter</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>CatalogueService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>catalogue, seating</t>
+          <t>platform-ops, tenancy</t>
         </is>
       </c>
       <c r="D52" s="10" t="n">
@@ -3998,17 +3998,17 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>tenancy.data_retention_setting</t>
+          <t>seating.seat_reservation_item</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>TenancyService</t>
+          <t>CatalogueService</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>access, tenancy</t>
+          <t>catalogue, seating</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
@@ -4023,23 +4023,48 @@
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>pii.consent_identifier</t>
+          <t>tenancy.data_retention_setting</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>IdentityService</t>
+          <t>TenancyService</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>identity, marketing-crm</t>
+          <t>access, tenancy</t>
         </is>
       </c>
       <c r="D54" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>Checked and correct — a side effect of the writing service's own job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>pii.consent_identifier</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>IdentityService</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>identity, marketing-crm</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>Checked and correct — a side effect of the writing service's own job.</t>
         </is>

</xml_diff>